<commit_message>
update manage location clusters v1
</commit_message>
<xml_diff>
--- a/assets/manage-location-clusters-template.xlsx
+++ b/assets/manage-location-clusters-template.xlsx
@@ -219,12 +219,22 @@
 <file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
-    <author>RongViet</author>
+    <author>RVF</author>
   </authors>
   <commentList>
-    <comment ref="G1" authorId="0" shapeId="0">
+    <comment ref="E1" authorId="0" shapeId="0">
       <text>
-        <t>Copy slug từ sheet 'Hướng dẫn &amp; Danh mục'. Nhiều môn ngăn bằng dấu phẩy, không dấu cách. VD: cau-long-don,tennis-don</t>
+        <t>Tên Tỉnh/Thành — dùng để lọc danh sách. Khớp đúng tên để mapping bộ lọc. VD: Đà Nẵng</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>Tên Xã/Phường thuộc Tỉnh/Thành ở cột trước. VD: Hòa Xuân</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>Copy slug từ sheet 'Hướng dẫn &amp; Danh mục'. Nhiều môn ngăn bằng dấu phẩy. VD: cau-long-don,tennis-don</t>
       </text>
     </comment>
   </commentList>
@@ -579,6 +589,13 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>6. Cột 'Tỉnh/Thành' &amp; 'Xã/Phường' (không bắt buộc) — nhập đúng tên để lọc danh sách theo khu vực; bỏ trống vẫn import được.</t>
+        </is>
+      </c>
+    </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
@@ -592,9 +609,6 @@
           <t>• Nhập SLUG (cột trái), KHÔNG nhập tên tiếng Việt.   VD đúng:  cau-long-don</t>
         </is>
       </c>
-      <c r="B11" s="6" t="n"/>
-      <c r="C11" s="6" t="n"/>
-      <c r="D11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -602,9 +616,6 @@
           <t>• Nhiều môn: ngăn nhau bằng dấu phẩy, KHÔNG dấu cách.   VD:  cau-long-don,tennis-don</t>
         </is>
       </c>
-      <c r="B12" s="6" t="n"/>
-      <c r="C12" s="6" t="n"/>
-      <c r="D12" s="6" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -612,9 +623,6 @@
           <t>• Slug sai / không có trong danh sách =&gt; dòng đó bị TỪ CHỐI khi import.</t>
         </is>
       </c>
-      <c r="B13" s="6" t="n"/>
-      <c r="C13" s="6" t="n"/>
-      <c r="D13" s="6" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
@@ -1033,7 +1041,8 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="17">
+    <mergeCell ref="A9:H9"/>
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="A38:B38"/>
     <mergeCell ref="A7:H7"/>
@@ -1062,19 +1071,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:M24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
     <col width="28" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
     <col width="22" customWidth="1" min="10" max="10"/>
     <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1100,30 +1111,39 @@
       </c>
       <c r="E1" s="12" t="inlineStr">
         <is>
+          <t>Tỉnh/Thành (province)</t>
+        </is>
+      </c>
+      <c r="F1" s="12" t="inlineStr">
+        <is>
+          <t>Xã/Phường (ward)</t>
+        </is>
+      </c>
+      <c r="G1" s="12" t="inlineStr">
+        <is>
           <t>Vĩ độ (latitude)</t>
         </is>
       </c>
-      <c r="F1" s="12" t="inlineStr">
+      <c r="H1" s="12" t="inlineStr">
         <is>
           <t>Kinh độ (longitude)</t>
         </is>
       </c>
-      <c r="G1" s="12" t="inlineStr">
+      <c r="I1" s="12" t="inlineStr">
         <is>
           <t>Môn (sports) *</t>
         </is>
       </c>
-      <c r="H1" s="12" t="inlineStr">
+      <c r="J1" s="12" t="inlineStr">
         <is>
           <t>Kích hoạt (is_active)</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="L1" s="4" t="inlineStr">
         <is>
           <t>📌 SPORTS — COPY SLUG, KHÔNG TỰ GÕ</t>
         </is>
       </c>
-      <c r="K1" s="13" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
@@ -1146,23 +1166,33 @@
           <t>Hòa Xuân, Đà Nẵng</t>
         </is>
       </c>
-      <c r="E2" s="14" t="n">
+      <c r="E2" s="14" t="inlineStr">
+        <is>
+          <t>Đà Nẵng</t>
+        </is>
+      </c>
+      <c r="F2" s="14" t="inlineStr">
+        <is>
+          <t>Hòa Xuân</t>
+        </is>
+      </c>
+      <c r="G2" s="14" t="n">
         <v>16.0312</v>
       </c>
-      <c r="F2" s="14" t="n">
+      <c r="H2" s="14" t="n">
         <v>108.2249</v>
       </c>
-      <c r="G2" s="14" t="inlineStr">
+      <c r="I2" s="14" t="inlineStr">
         <is>
           <t>cau-long-don,cau-long-doi</t>
         </is>
       </c>
-      <c r="H2" s="14" t="inlineStr">
+      <c r="J2" s="14" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="J2" s="15" t="inlineStr">
+      <c r="L2" s="15" t="inlineStr">
         <is>
           <t>Nhiều môn ngăn bằng dấu phẩy. VD: cau-long-don,tennis-don</t>
         </is>
@@ -1185,280 +1215,290 @@
           <t>TP Buôn Ma Thuột, Đắk Lắk</t>
         </is>
       </c>
-      <c r="E3" s="14" t="n">
+      <c r="E3" s="14" t="inlineStr">
+        <is>
+          <t>Đắk Lắk</t>
+        </is>
+      </c>
+      <c r="F3" s="14" t="inlineStr">
+        <is>
+          <t>Tân Lập</t>
+        </is>
+      </c>
+      <c r="G3" s="14" t="n">
         <v>12.679</v>
       </c>
-      <c r="F3" s="14" t="n">
+      <c r="H3" s="14" t="n">
         <v>108.05</v>
       </c>
-      <c r="G3" s="14" t="inlineStr">
+      <c r="I3" s="14" t="inlineStr">
         <is>
           <t>bong-ban-don</t>
         </is>
       </c>
-      <c r="H3" s="14" t="inlineStr">
+      <c r="J3" s="14" t="inlineStr">
         <is>
           <t>TRUE</t>
         </is>
       </c>
-      <c r="J3" s="16" t="inlineStr">
+      <c r="L3" s="16" t="inlineStr">
         <is>
           <t>slug</t>
         </is>
       </c>
-      <c r="K3" s="16" t="inlineStr">
+      <c r="M3" s="16" t="inlineStr">
         <is>
           <t>Tên môn</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="J4" s="17" t="inlineStr">
+      <c r="L4" s="17" t="inlineStr">
         <is>
           <t>bong-ban-don</t>
         </is>
       </c>
-      <c r="K4" s="9" t="inlineStr">
+      <c r="M4" s="9" t="inlineStr">
         <is>
           <t>Bóng bàn đơn</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="J5" s="17" t="inlineStr">
+      <c r="L5" s="17" t="inlineStr">
         <is>
           <t>bong-chuyen</t>
         </is>
       </c>
-      <c r="K5" s="9" t="inlineStr">
+      <c r="M5" s="9" t="inlineStr">
         <is>
           <t>Bóng chuyền</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="J6" s="17" t="inlineStr">
+      <c r="L6" s="17" t="inlineStr">
         <is>
           <t>bong-da</t>
         </is>
       </c>
-      <c r="K6" s="9" t="inlineStr">
+      <c r="M6" s="9" t="inlineStr">
         <is>
           <t>Bóng đá</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="J7" s="17" t="inlineStr">
+      <c r="L7" s="17" t="inlineStr">
         <is>
           <t>bong-da-5</t>
         </is>
       </c>
-      <c r="K7" s="9" t="inlineStr">
+      <c r="M7" s="9" t="inlineStr">
         <is>
           <t>Bóng đá 5 người</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="J8" s="17" t="inlineStr">
+      <c r="L8" s="17" t="inlineStr">
         <is>
           <t>bong-da-7</t>
         </is>
       </c>
-      <c r="K8" s="9" t="inlineStr">
+      <c r="M8" s="9" t="inlineStr">
         <is>
           <t>Bóng đá 7 người</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="J9" s="17" t="inlineStr">
+      <c r="L9" s="17" t="inlineStr">
         <is>
           <t>bong-da-mini-league</t>
         </is>
       </c>
-      <c r="K9" s="9" t="inlineStr">
+      <c r="M9" s="9" t="inlineStr">
         <is>
           <t>Bóng đá Mini League</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="J10" s="17" t="inlineStr">
+      <c r="L10" s="17" t="inlineStr">
         <is>
           <t>bong-ro-3x3</t>
         </is>
       </c>
-      <c r="K10" s="9" t="inlineStr">
+      <c r="M10" s="9" t="inlineStr">
         <is>
           <t>Bóng rổ 3x3</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="J11" s="17" t="inlineStr">
+      <c r="L11" s="17" t="inlineStr">
         <is>
           <t>bong-ro-5x5</t>
         </is>
       </c>
-      <c r="K11" s="9" t="inlineStr">
+      <c r="M11" s="9" t="inlineStr">
         <is>
           <t>Bóng rổ 5x5</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="J12" s="17" t="inlineStr">
+      <c r="L12" s="17" t="inlineStr">
         <is>
           <t>cau-long-doi</t>
         </is>
       </c>
-      <c r="K12" s="9" t="inlineStr">
+      <c r="M12" s="9" t="inlineStr">
         <is>
           <t>Cầu lông đôi</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="J13" s="17" t="inlineStr">
+      <c r="L13" s="17" t="inlineStr">
         <is>
           <t>cau-long-don</t>
         </is>
       </c>
-      <c r="K13" s="9" t="inlineStr">
+      <c r="M13" s="9" t="inlineStr">
         <is>
           <t>Cầu lông đơn</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="J14" s="17" t="inlineStr">
+      <c r="L14" s="17" t="inlineStr">
         <is>
           <t>co-vua</t>
         </is>
       </c>
-      <c r="K14" s="9" t="inlineStr">
+      <c r="M14" s="9" t="inlineStr">
         <is>
           <t>Cờ vua</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="J15" s="17" t="inlineStr">
+      <c r="L15" s="17" t="inlineStr">
         <is>
           <t>esport-1v1</t>
         </is>
       </c>
-      <c r="K15" s="9" t="inlineStr">
+      <c r="M15" s="9" t="inlineStr">
         <is>
           <t>Esport 1v1</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="J16" s="17" t="inlineStr">
+      <c r="L16" s="17" t="inlineStr">
         <is>
           <t>fps-solo</t>
         </is>
       </c>
-      <c r="K16" s="9" t="inlineStr">
+      <c r="M16" s="9" t="inlineStr">
         <is>
           <t>FPS Solo</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="J17" s="17" t="inlineStr">
+      <c r="L17" s="17" t="inlineStr">
         <is>
           <t>fps-team</t>
         </is>
       </c>
-      <c r="K17" s="9" t="inlineStr">
+      <c r="M17" s="9" t="inlineStr">
         <is>
           <t>FPS Team</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="J18" s="17" t="inlineStr">
+      <c r="L18" s="17" t="inlineStr">
         <is>
           <t>moba-3v3</t>
         </is>
       </c>
-      <c r="K18" s="9" t="inlineStr">
+      <c r="M18" s="9" t="inlineStr">
         <is>
           <t>MOBA 3v3</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="J19" s="17" t="inlineStr">
+      <c r="L19" s="17" t="inlineStr">
         <is>
           <t>moba-5v5</t>
         </is>
       </c>
-      <c r="K19" s="9" t="inlineStr">
+      <c r="M19" s="9" t="inlineStr">
         <is>
           <t>MOBA 5v5</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="J20" s="17" t="inlineStr">
+      <c r="L20" s="17" t="inlineStr">
         <is>
           <t>moba-league</t>
         </is>
       </c>
-      <c r="K20" s="9" t="inlineStr">
+      <c r="M20" s="9" t="inlineStr">
         <is>
           <t>MOBA League</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="J21" s="17" t="inlineStr">
+      <c r="L21" s="17" t="inlineStr">
         <is>
           <t>phong-trao</t>
         </is>
       </c>
-      <c r="K21" s="9" t="inlineStr">
+      <c r="M21" s="9" t="inlineStr">
         <is>
           <t>Phong Trào</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="J22" s="17" t="inlineStr">
+      <c r="L22" s="17" t="inlineStr">
         <is>
           <t>squash</t>
         </is>
       </c>
-      <c r="K22" s="9" t="inlineStr">
+      <c r="M22" s="9" t="inlineStr">
         <is>
           <t>Squash</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="J23" s="17" t="inlineStr">
+      <c r="L23" s="17" t="inlineStr">
         <is>
           <t>tennis-doi</t>
         </is>
       </c>
-      <c r="K23" s="9" t="inlineStr">
+      <c r="M23" s="9" t="inlineStr">
         <is>
           <t>Tennis (đôi)</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="J24" s="17" t="inlineStr">
+      <c r="L24" s="17" t="inlineStr">
         <is>
           <t>tennis-don</t>
         </is>
       </c>
-      <c r="K24" s="9" t="inlineStr">
+      <c r="M24" s="9" t="inlineStr">
         <is>
           <t>Tennis (đơn)</t>
         </is>
@@ -1466,11 +1506,11 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="J1:K1"/>
-    <mergeCell ref="J2:K2"/>
+    <mergeCell ref="L1:M1"/>
+    <mergeCell ref="L2:M2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="H2:H500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>